<commit_message>
export backlogWh, change template
</commit_message>
<xml_diff>
--- a/src/main/resources/assets/template/ExportBacklogWhTemplate.xlsx
+++ b/src/main/resources/assets/template/ExportBacklogWhTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Backend\kvc-wh-be\src\main\resources\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C09169-4838-4EB5-849A-599D26B112AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1466668F-ADC3-42EF-B610-2CAE2E650471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1710" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,18 +25,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>BIN</t>
-  </si>
-  <si>
-    <t>PO</t>
-  </si>
-  <si>
-    <t>RECEIVING DATE</t>
-  </si>
-  <si>
-    <t>QTY</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>Mã gói</t>
+  </si>
+  <si>
+    <t>Số PO</t>
+  </si>
+  <si>
+    <t>BIN#</t>
+  </si>
+  <si>
+    <t>Số lượng</t>
+  </si>
+  <si>
+    <t>Số thùng</t>
+  </si>
+  <si>
+    <t>Ngày nhận hàng</t>
+  </si>
+  <si>
+    <t>Ngày Insp</t>
   </si>
 </sst>
 </file>
@@ -44,7 +53,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -96,19 +105,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,27 +402,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.21875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="20" style="5" customWidth="1"/>
-    <col min="4" max="4" width="28.5546875" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" style="3" customWidth="1"/>
+    <col min="3" max="4" width="25" style="5" customWidth="1"/>
+    <col min="5" max="5" width="20" style="5" customWidth="1"/>
+    <col min="6" max="6" width="21.44140625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
exclude 50xxx location when import amoeba backlog, add itemname column when export backlog
</commit_message>
<xml_diff>
--- a/src/main/resources/assets/template/ExportBacklogWhTemplate.xlsx
+++ b/src/main/resources/assets/template/ExportBacklogWhTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Backend\kvc-wh-be\src\main\resources\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\resources\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1466668F-ADC3-42EF-B610-2CAE2E650471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66AD687A-3324-4116-9B9B-49197DFD00F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1710" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28830" yWindow="2880" windowWidth="21600" windowHeight="11175" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tồn kho" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Mã gói</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>Ngày Insp</t>
+  </si>
+  <si>
+    <t>Tên NVL</t>
   </si>
 </sst>
 </file>
@@ -105,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -118,10 +121,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,18 +401,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="22.44140625" style="3" customWidth="1"/>
-    <col min="3" max="4" width="25" style="5" customWidth="1"/>
-    <col min="5" max="5" width="20" style="5" customWidth="1"/>
-    <col min="6" max="6" width="21.44140625" style="7" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="3" customWidth="1"/>
+    <col min="3" max="5" width="25" style="5" customWidth="1"/>
+    <col min="6" max="6" width="20" style="5" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -427,12 +426,15 @@
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add lot no and issue to inquiry and download backlog wh, system stock taking
</commit_message>
<xml_diff>
--- a/src/main/resources/assets/template/ExportBacklogWhTemplate.xlsx
+++ b/src/main/resources/assets/template/ExportBacklogWhTemplate.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\resources\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66AD687A-3324-4116-9B9B-49197DFD00F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2189ABE6-F025-4C6C-AA5A-A6963E4A369F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28830" yWindow="2880" windowWidth="21600" windowHeight="11175" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tồn kho" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Mã gói</t>
   </si>
@@ -49,6 +49,12 @@
   </si>
   <si>
     <t>Tên NVL</t>
+  </si>
+  <si>
+    <t>Số lô</t>
+  </si>
+  <si>
+    <t>Ngày sản xuất</t>
   </si>
 </sst>
 </file>
@@ -401,18 +407,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.42578125" style="3" customWidth="1"/>
     <col min="2" max="2" width="22.42578125" style="3" customWidth="1"/>
-    <col min="3" max="5" width="25" style="5" customWidth="1"/>
-    <col min="6" max="6" width="20" style="5" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" customWidth="1"/>
+    <col min="3" max="7" width="25" style="5" customWidth="1"/>
+    <col min="8" max="8" width="20" style="5" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -429,12 +435,18 @@
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>